<commit_message>
Remove the update_records_list_adding_ml_noises_v7.sh script as it is no longer needed. The script contained various commented-out Python commands for processing Excel files and applying machine learning noise, which have been deprecated.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui_1024_0_5_0_7_test_0_12.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui_1024_0_5_0_7_test_0_12.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="380" yWindow="380" windowWidth="18600" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="600" yWindow="1140" windowWidth="18600" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="13.6328125" customWidth="1" style="13" min="3" max="3"/>
@@ -547,16 +547,16 @@
     <col width="4.90625" customWidth="1" min="16" max="16"/>
     <col width="8.90625" customWidth="1" min="17" max="17"/>
     <col width="9.26953125" customWidth="1" min="18" max="18"/>
-    <col width="9.7265625" customWidth="1" style="9" min="19" max="19"/>
-    <col width="9.81640625" customWidth="1" min="20" max="20"/>
-    <col width="13.1796875" customWidth="1" min="21" max="21"/>
-    <col width="12.08984375" customWidth="1" style="10" min="22" max="22"/>
-    <col width="54.6328125" customWidth="1" min="23" max="23"/>
-    <col width="28.81640625" customWidth="1" min="24" max="24"/>
-    <col width="27.1796875" customWidth="1" min="25" max="25"/>
-    <col width="13.6328125" customWidth="1" style="5" min="26" max="31"/>
-    <col width="13.6328125" customWidth="1" min="32" max="32"/>
-    <col width="8.7265625" customWidth="1" min="33" max="48"/>
+    <col width="9.7265625" customWidth="1" style="9" min="19" max="23"/>
+    <col hidden="1" width="9.81640625" customWidth="1" min="24" max="24"/>
+    <col hidden="1" width="13.1796875" customWidth="1" min="25" max="25"/>
+    <col hidden="1" width="12.08984375" customWidth="1" style="10" min="26" max="26"/>
+    <col width="54.6328125" customWidth="1" min="27" max="27"/>
+    <col width="28.81640625" customWidth="1" min="28" max="28"/>
+    <col width="27.1796875" customWidth="1" min="29" max="29"/>
+    <col width="13.6328125" customWidth="1" style="5" min="30" max="35"/>
+    <col width="13.6328125" customWidth="1" min="36" max="36"/>
+    <col width="8.7265625" customWidth="1" min="37" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -655,40 +655,59 @@
           <t>h_nz_frac%</t>
         </is>
       </c>
-      <c r="T1" s="11" t="n"/>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> out</t>
+        </is>
+      </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>rdr</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>noi</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>tp%</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>ml_nz_cnt</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>ml_nz_len</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>ml_nz_frac%</t>
+        </is>
+      </c>
+      <c r="AA1" s="11" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>recordingId</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>userId</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
-        </is>
-      </c>
-      <c r="X1" s="7" t="inlineStr">
-        <is>
-          <t>out</t>
-        </is>
-      </c>
-      <c r="Y1" s="7" t="inlineStr">
-        <is>
-          <t>rdr</t>
-        </is>
-      </c>
-      <c r="Z1" s="7" t="inlineStr">
-        <is>
-          <t>noi</t>
-        </is>
-      </c>
-      <c r="AA1" s="7" t="inlineStr">
-        <is>
-          <t>ml_nz_frac%</t>
         </is>
       </c>
     </row>
@@ -760,37 +779,46 @@
       <c r="S2" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>EXTERNALLY_ANNOTATED,FOR_EXTERNAL_ANNOTATING,PSEUDO_ANNOTATED</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="T2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W2" s="9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="X2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>60f945e187cf66e97e37810e</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>6034c808d6c2740008035ede</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr">
+      <c r="AD2" s="5" t="inlineStr">
         <is>
           <t>Truputi plaukioja amplitudė</t>
         </is>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>17.2</v>
       </c>
     </row>
     <row r="3">
@@ -859,37 +887,46 @@
       <c r="S3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>EXTERNALLY_ANNOTATED,FOR_EXTERNAL_ANNOTATING,PSEUDO_ANNOTATED</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
+      <c r="T3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="W3" s="9" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="X3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>PSEUDO_ANNOTATED</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>615516b62312e50c3f168e38</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>6034c808d6c2740008035ede</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="AD3" s="5" t="inlineStr">
         <is>
           <t>Labai ilgas, &gt; 4000. Praleistas pikas, gydytojas pažymėjo. Kokybė nėra aiški</t>
         </is>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>86.7</v>
       </c>
     </row>
     <row r="4">
@@ -958,37 +995,46 @@
       <c r="S4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="W4" s="9" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="X4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>60a92aa454352a03116dc1f5</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="AD4" s="5" t="inlineStr">
         <is>
           <t>keliasdešimt sekundžių pradžia nenusistovėjusi, izolinija, nemažai pašokinėja, pasitaiko nedideli raumenų triukšmai,  10 pūpsnių triukšmo intervalas ties 488800, 608300, 693800, 703000, 855000,860600,864600, 867100, 876800, kažkokie triukšmai  užsideda ant izolinijos pabaigoje</t>
         </is>
-      </c>
-      <c r="X4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>54.4</v>
       </c>
     </row>
     <row r="5">
@@ -1059,37 +1105,46 @@
       <c r="S5" s="9" t="n">
         <v>6.5</v>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>EXTERNALLY_ANNOTATED,FOR_EXTERNAL_ANNOTATING,PSEUDO_ANNOTATED</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
+      <c r="T5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="W5" s="9" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="X5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>PSEUDO_ANNOTATED</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>60efffba87cf660aac377fe7</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="AD5" s="5" t="inlineStr">
         <is>
           <t>Yra S. Nedidelis, bet pastovus  BW, yra epizodų su EMG</t>
         </is>
-      </c>
-      <c r="X5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>72.09999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -1158,37 +1213,46 @@
       <c r="S6" s="9" t="n">
         <v>2.4</v>
       </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
+      <c r="T6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="W6" s="9" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="X6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; FOR_EXTERNAL_ANNOTATING</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
         <is>
           <t>60f9188487cf669c7e3780b8</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr">
+      <c r="AD6" s="5" t="inlineStr">
         <is>
           <t>izolinija šokinėja nedaug, vietomis išlenda raumenų triušmai. Kokybė nebloga, žymėjimas koreguotas, gana daug triukšminių intervalų, gal geriau tinka testavimui</t>
         </is>
-      </c>
-      <c r="X6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>36.8</v>
       </c>
     </row>
     <row r="7">
@@ -1254,37 +1318,46 @@
       <c r="S7" s="9" t="n">
         <v>3.3</v>
       </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>EXTERNALLY_ANNOTATED,FOR_EXTERNAL_ANNOTATING,PSEUDO_ANNOTATED</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
+      <c r="T7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" s="9" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="X7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>PSEUDO_ANNOTATED</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
         <is>
           <t>60f9188487cf6632713780c5</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W7" s="6" t="inlineStr">
+      <c r="AD7" s="6" t="inlineStr">
         <is>
           <t>Paskutinės 16 sekundžių diržas nuimtas</t>
         </is>
-      </c>
-      <c r="X7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>7.1</v>
       </c>
     </row>
     <row r="8">
@@ -1348,37 +1421,46 @@
       <c r="S8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
+      <c r="T8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="W8" s="9" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="X8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; FOR_EXTERNAL_ANNOTATING</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>60f9188487cf66240e3780bf</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W8" s="5" t="inlineStr">
+      <c r="AD8" s="5" t="inlineStr">
         <is>
           <t>Neaišku, kas yra ties 12300 klausimas gydytojui. Gal verta užblokuoti 3 pūpsnius pradedant reikšme 68100, gal dar 2 - ties 92700, nors dabartiniam ML nepakenkė. Kokybė nebloga, žymėjimas koreguotas , tačiau nors triukšmai pažymėti, bet vis tiek dar išlenda silpni raumenų triukšmai, mokymui nerekomenduojamas</t>
         </is>
-      </c>
-      <c r="X8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>50.6</v>
       </c>
     </row>
     <row r="9">
@@ -1447,32 +1529,41 @@
       <c r="S9" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="T9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; NOISES_ANNOTATED; AI_DATASET</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>638d8f609e4d4309eebbb0f1</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
-      </c>
-      <c r="X9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1536,37 +1627,46 @@
       <c r="S10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
+      <c r="T10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="W10" s="9" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="X10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; FOR_EXTERNAL_ANNOTATING</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>638d8e519e4d43245abbb0c5</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
+      <c r="AD10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Švarumo lygis didžojoje dalyje arti 10, tačiau apie vidurį yra ilgas fragmentas su nežymėtu silpnu# raumenų triukšmu. Žymėjimas koreguotas, dėl įtraukimo į mokymo grupę, abejotina </t>
         </is>
-      </c>
-      <c r="X10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>42.8</v>
       </c>
     </row>
     <row r="11">
@@ -1635,32 +1735,41 @@
       <c r="S11" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
+      <c r="T11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W11" s="9" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="X11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; NOISES_ANNOTATED; AI_DATASET</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>638d8f5d9e4d43301ebbb0df</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
-      </c>
-      <c r="X11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>14.6</v>
       </c>
     </row>
     <row r="12">
@@ -1726,32 +1835,41 @@
       <c r="S12" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W12" s="9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="X12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="inlineStr">
         <is>
           <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="AB12" t="inlineStr">
         <is>
           <t>613f57ea3d08d45609cdcc86</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>613b1bc63d08d41309cdc8f1</t>
         </is>
-      </c>
-      <c r="X12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>14.3</v>
       </c>
     </row>
     <row r="13">
@@ -1800,29 +1918,43 @@
       <c r="S13" s="9" t="n">
         <v>2.6</v>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="T13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" s="9" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="X13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; FOR_EXTERNAL_ANNOTATING</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>60f9188487cf6678b43780c3</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>60a917b354352a3df86dc1f2</t>
         </is>
       </c>
-      <c r="W13" s="5" t="n"/>
-      <c r="X13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>26.4</v>
-      </c>
+      <c r="AD13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1875,29 +2007,43 @@
       <c r="S14" s="9" t="n">
         <v>7.6</v>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="T14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W14" s="9" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="X14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>FULLY_ANNOTATED_PROFESSIONALLY; NOISES_ANNOTATED; AI_DATASET</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
         <is>
           <t>67bad7b24cf53e79dfed20fb</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>607efbd094e6ea3b5a1ab959</t>
         </is>
       </c>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>41.2</v>
-      </c>
+      <c r="AD14" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>